<commit_message>
Give four of the new Section 1 questions their own data
I reused the North/South/Creek/Home/Rented farm across six questions. Q18's
yields and Q25's yields-and-acres were Q1's exactly, so a student who had
drawn Q1 could read intermediate values straight off its answer workbook --
the same defect that was fixed in Q5 several rounds ago, reintroduced by me
while writing the new questions.

Q12, Q17, Q18 and Q25 now carry distinct datasets, and their answer keys and
workbooks are recomputed to match. No two questions in Section 1 now share
more than 70% of their numbers.

Found by checking dataset overlap across all thirty questions rather than by
reading them, which is the only way this kind of thing shows up.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0165WQeoaB3CPsnpvD7o3Yah
</commit_message>
<xml_diff>
--- a/practice/answers/s1_q12.xlsx
+++ b/practice/answers/s1_q12.xlsx
@@ -526,17 +526,17 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>North</t>
+          <t>Birch</t>
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>41.2</v>
+        <v>46.9</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>South</t>
+          <t>Coulee</t>
         </is>
       </c>
       <c r="B6" s="5" t="n"/>
@@ -544,17 +544,17 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Creek</t>
+          <t>Draw</t>
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>44.8</v>
+        <v>52.7</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Home</t>
+          <t>Flats</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -566,17 +566,17 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Rented</t>
+          <t>Gully</t>
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>39.9</v>
+        <v>44.3</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Quarter</t>
+          <t>Hollow</t>
         </is>
       </c>
       <c r="B10" s="5" t="n"/>
@@ -661,7 +661,7 @@
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>COUNT 3, COUNTA 4 -- the difference is the words 'not seeded'. The average is 41.97 over three values. Type 0 into the two blanks and it falls to 25.18, which asserts those fields yielded nothing.</t>
+          <t>COUNT 3, COUNTA 4 -- the difference is the words 'not seeded'. The average is 47.97 over three values. Type 0 into the two blanks and it falls to 28.78, which asserts those fields yielded nothing.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Six crops, not seven
</commit_message>
<xml_diff>
--- a/practice/answers/s1_q12.xlsx
+++ b/practice/answers/s1_q12.xlsx
@@ -16,9 +16,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.0"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="8">
     <font>
       <name val="Calibri"/>
@@ -46,12 +44,12 @@
     </font>
     <font>
       <name val="Arial"/>
+      <b val="1"/>
       <color rgb="0024302A"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
-      <b val="1"/>
       <color rgb="0024302A"/>
       <sz val="10"/>
     </font>
@@ -96,7 +94,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -107,20 +105,14 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -487,26 +479,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="18" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Blanks, text, and what the functions count</t>
+          <t>One SUM, three blocks</t>
         </is>
       </c>
     </row>
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>COUNT sees numbers, COUNTA sees anything typed, AVERAGE skips both blanks and text. Filling the blanks with zero would change the claim being made.</t>
+          <t>A range that spans the blank rows happens to give the right answer here. Naming the three ranges says what the total is actually made of.</t>
         </is>
       </c>
     </row>
@@ -514,162 +506,192 @@
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Field</t>
+          <t>Parcel</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Yield (bu/ac)</t>
+          <t>Acres</t>
         </is>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Birch</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="n">
-        <v>46.9</v>
+          <t>Home quarter</t>
+        </is>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>Coulee</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="n"/>
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>NW</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>142</v>
+      </c>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Draw</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="n">
-        <v>52.7</v>
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>SW</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>318</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>Flats</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>not seeded</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Gully</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="n">
-        <v>44.3</v>
-      </c>
-    </row>
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>NE</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1"/>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Hollow</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="n"/>
-    </row>
-    <row r="11" ht="18" customHeight="1"/>
+          <t>River section</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>North strip</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="n">
+        <v>205</v>
+      </c>
+    </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>COUNT (numbers)</t>
-        </is>
-      </c>
-      <c r="C12" s="8">
-        <f>COUNT(B5:B10)</f>
-        <v/>
-      </c>
-      <c r="D12" s="9">
-        <f>_xlfn.FORMULATEXT(C12)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>COUNTA (anything)</t>
-        </is>
-      </c>
-      <c r="C13" s="8">
-        <f>COUNTA(B5:B10)</f>
-        <v/>
-      </c>
-      <c r="D13" s="9">
-        <f>_xlfn.FORMULATEXT(C13)</f>
-        <v/>
-      </c>
-    </row>
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>South strip</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="n">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1"/>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>SUM</t>
-        </is>
-      </c>
-      <c r="C14" s="10">
-        <f>SUM(B5:B10)</f>
-        <v/>
-      </c>
-      <c r="D14" s="9">
-        <f>_xlfn.FORMULATEXT(C14)</f>
-        <v/>
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>East lease</t>
+        </is>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>AVERAGE</t>
-        </is>
-      </c>
-      <c r="C15" s="11">
-        <f>AVERAGE(B5:B10)</f>
-        <v/>
-      </c>
-      <c r="D15" s="9">
-        <f>_xlfn.FORMULATEXT(C15)</f>
-        <v/>
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Field 1</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="n">
+        <v>264</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>SUM / COUNT</t>
-        </is>
-      </c>
-      <c r="C16" s="11">
-        <f>SUM(B5:B10)/COUNT(B5:B10)</f>
-        <v/>
-      </c>
-      <c r="D16" s="9">
-        <f>_xlfn.FORMULATEXT(C16)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" ht="18" customHeight="1"/>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="12" t="inlineStr">
-        <is>
-          <t>COUNT 3, COUNTA 4 -- the difference is the words 'not seeded'. The average is 47.97 over three values. Type 0 into the two blanks and it falls to 28.78, which asserts those fields yielded nothing.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="18" customHeight="1"/>
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Field 2</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="n">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Field 3</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="n">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1"/>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>One range, first to last</t>
+        </is>
+      </c>
+      <c r="C19" s="8">
+        <f>SUM(B6:B17)</f>
+        <v/>
+      </c>
+      <c r="D19" s="9">
+        <f>_xlfn.FORMULATEXT(C19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>The three ranges named</t>
+        </is>
+      </c>
+      <c r="C20" s="8">
+        <f>SUM(B6:B8,B11:B12,B15:B17)</f>
+        <v/>
+      </c>
+      <c r="D20" s="9">
+        <f>_xlfn.FORMULATEXT(C20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>...plus a 60-acre rental</t>
+        </is>
+      </c>
+      <c r="C21" s="8">
+        <f>SUM(B6:B8,B11:B12,B15:B17,60)</f>
+        <v/>
+      </c>
+      <c r="D21" s="9">
+        <f>_xlfn.FORMULATEXT(C21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>The first block only</t>
+        </is>
+      </c>
+      <c r="C22" s="8">
+        <f>SUM(B6:B8)</f>
+        <v/>
+      </c>
+      <c r="D22" s="9">
+        <f>_xlfn.FORMULATEXT(C22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1"/>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>1,421 / 1,421 / 1,481 / 556. The first two agree only because nothing unwanted sits between the first acreage and the last. Put a subtotal in one of those blank rows and the single range swallows it without a word.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A24:D24"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>